<commit_message>
Refresh JFK risk analysis for multi-year data
</commit_message>
<xml_diff>
--- a/data/processed/jfk_airline_risk_profile.xlsx
+++ b/data/processed/jfk_airline_risk_profile.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -495,43 +495,43 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3780</v>
+        <v>19500</v>
       </c>
       <c r="C2" t="n">
-        <v>1096</v>
+        <v>4451</v>
       </c>
       <c r="D2" t="n">
-        <v>55</v>
+        <v>391</v>
       </c>
       <c r="E2" t="n">
-        <v>33</v>
+        <v>100</v>
       </c>
       <c r="F2" t="n">
-        <v>59777</v>
+        <v>239570</v>
       </c>
       <c r="G2" t="n">
-        <v>11984</v>
+        <v>62682</v>
       </c>
       <c r="H2" t="n">
-        <v>3572</v>
+        <v>17620</v>
       </c>
       <c r="I2" t="n">
-        <v>34384</v>
+        <v>112471</v>
       </c>
       <c r="J2" t="n">
-        <v>310</v>
+        <v>799</v>
       </c>
       <c r="K2" t="n">
-        <v>9527</v>
+        <v>45998</v>
       </c>
       <c r="L2" t="n">
-        <v>0.28994708994709</v>
+        <v>0.2282564102564102</v>
       </c>
       <c r="M2" t="n">
-        <v>0.01455026455026455</v>
+        <v>0.02005128205128205</v>
       </c>
       <c r="N2" t="n">
-        <v>54.54105839416059</v>
+        <v>53.82385980678499</v>
       </c>
     </row>
     <row r="3">
@@ -541,43 +541,43 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>14266</v>
+        <v>76512</v>
       </c>
       <c r="C3" t="n">
-        <v>3432</v>
+        <v>16042</v>
       </c>
       <c r="D3" t="n">
-        <v>206</v>
+        <v>1768</v>
       </c>
       <c r="E3" t="n">
-        <v>73</v>
+        <v>290</v>
       </c>
       <c r="F3" t="n">
-        <v>305149</v>
+        <v>1337832</v>
       </c>
       <c r="G3" t="n">
-        <v>88461</v>
+        <v>482269</v>
       </c>
       <c r="H3" t="n">
-        <v>10691</v>
+        <v>62379</v>
       </c>
       <c r="I3" t="n">
-        <v>86956</v>
+        <v>300815</v>
       </c>
       <c r="J3" t="n">
-        <v>507</v>
+        <v>4916</v>
       </c>
       <c r="K3" t="n">
-        <v>118534</v>
+        <v>487453</v>
       </c>
       <c r="L3" t="n">
-        <v>0.2405719893452965</v>
+        <v>0.2096664575491426</v>
       </c>
       <c r="M3" t="n">
-        <v>0.01443992709939717</v>
+        <v>0.02310748640736094</v>
       </c>
       <c r="N3" t="n">
-        <v>88.91287878787878</v>
+        <v>83.39558658521382</v>
       </c>
     </row>
     <row r="4">
@@ -587,43 +587,43 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>30454</v>
+        <v>153673</v>
       </c>
       <c r="C4" t="n">
-        <v>6132</v>
+        <v>27882</v>
       </c>
       <c r="D4" t="n">
-        <v>421</v>
+        <v>3058</v>
       </c>
       <c r="E4" t="n">
-        <v>144</v>
+        <v>548</v>
       </c>
       <c r="F4" t="n">
-        <v>520793</v>
+        <v>2244825</v>
       </c>
       <c r="G4" t="n">
-        <v>194478</v>
+        <v>974305</v>
       </c>
       <c r="H4" t="n">
-        <v>27881</v>
+        <v>99535</v>
       </c>
       <c r="I4" t="n">
-        <v>160447</v>
+        <v>550237</v>
       </c>
       <c r="J4" t="n">
-        <v>281</v>
+        <v>4313</v>
       </c>
       <c r="K4" t="n">
-        <v>137706</v>
+        <v>616435</v>
       </c>
       <c r="L4" t="n">
-        <v>0.2013528600512248</v>
+        <v>0.1814372075771281</v>
       </c>
       <c r="M4" t="n">
-        <v>0.01382412819334078</v>
+        <v>0.01989939677106584</v>
       </c>
       <c r="N4" t="n">
-        <v>84.93036529680366</v>
+        <v>80.51162040025824</v>
       </c>
     </row>
     <row r="5">
@@ -633,258 +633,258 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>20342</v>
+        <v>96017</v>
       </c>
       <c r="C5" t="n">
-        <v>4173</v>
+        <v>14815</v>
       </c>
       <c r="D5" t="n">
-        <v>858</v>
+        <v>3690</v>
       </c>
       <c r="E5" t="n">
-        <v>16</v>
+        <v>110</v>
       </c>
       <c r="F5" t="n">
-        <v>405529</v>
+        <v>1320399</v>
       </c>
       <c r="G5" t="n">
-        <v>97354</v>
+        <v>362735</v>
       </c>
       <c r="H5" t="n">
-        <v>22966</v>
+        <v>87071</v>
       </c>
       <c r="I5" t="n">
-        <v>140211</v>
+        <v>442865</v>
       </c>
       <c r="J5" t="n">
-        <v>210</v>
+        <v>567</v>
       </c>
       <c r="K5" t="n">
-        <v>144788</v>
+        <v>427161</v>
       </c>
       <c r="L5" t="n">
-        <v>0.205142070592862</v>
+        <v>0.154295593488653</v>
       </c>
       <c r="M5" t="n">
-        <v>0.04217874348638286</v>
+        <v>0.0384306945645042</v>
       </c>
       <c r="N5" t="n">
-        <v>97.17924754373352</v>
+        <v>89.12581842726966</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Frontier Airlines</t>
+          <t>Envoy Air</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3166</v>
+        <v>932</v>
       </c>
       <c r="C6" t="n">
-        <v>745</v>
+        <v>104</v>
       </c>
       <c r="D6" t="n">
-        <v>41</v>
+        <v>99</v>
       </c>
       <c r="E6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>53862</v>
+        <v>9428</v>
       </c>
       <c r="G6" t="n">
-        <v>21225</v>
+        <v>2746</v>
       </c>
       <c r="H6" t="n">
-        <v>1499</v>
+        <v>128</v>
       </c>
       <c r="I6" t="n">
-        <v>10834</v>
+        <v>2882</v>
       </c>
       <c r="J6" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="K6" t="n">
-        <v>20304</v>
+        <v>3653</v>
       </c>
       <c r="L6" t="n">
-        <v>0.235312697409981</v>
+        <v>0.111587982832618</v>
       </c>
       <c r="M6" t="n">
-        <v>0.0129500947567909</v>
+        <v>0.1062231759656652</v>
       </c>
       <c r="N6" t="n">
-        <v>72.29798657718121</v>
+        <v>90.65384615384616</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Hawaiian Airlines</t>
+          <t>Frontier Airlines</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>365</v>
+        <v>3996</v>
       </c>
       <c r="C7" t="n">
-        <v>101</v>
+        <v>937</v>
       </c>
       <c r="D7" t="n">
+        <v>47</v>
+      </c>
+      <c r="E7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F7" t="n">
+        <v>65933</v>
+      </c>
+      <c r="G7" t="n">
+        <v>27442</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1638</v>
+      </c>
+      <c r="I7" t="n">
+        <v>12818</v>
+      </c>
+      <c r="J7" t="n">
         <v>0</v>
       </c>
-      <c r="E7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" t="n">
-        <v>4957</v>
-      </c>
-      <c r="G7" t="n">
-        <v>3492</v>
-      </c>
-      <c r="H7" t="n">
-        <v>301</v>
-      </c>
-      <c r="I7" t="n">
-        <v>164</v>
-      </c>
-      <c r="J7" t="n">
-        <v>63</v>
-      </c>
       <c r="K7" t="n">
-        <v>937</v>
+        <v>24035</v>
       </c>
       <c r="L7" t="n">
-        <v>0.2767123287671233</v>
+        <v>0.2344844844844845</v>
       </c>
       <c r="M7" t="n">
-        <v>0</v>
+        <v>0.01176176176176176</v>
       </c>
       <c r="N7" t="n">
-        <v>49.07920792079208</v>
+        <v>70.36606189967983</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>JetBlue Airways</t>
+          <t>Hawaiian Airlines</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>35874</v>
+        <v>1843</v>
       </c>
       <c r="C8" t="n">
-        <v>8287</v>
+        <v>644</v>
       </c>
       <c r="D8" t="n">
-        <v>848</v>
+        <v>7</v>
       </c>
       <c r="E8" t="n">
-        <v>95</v>
+        <v>10</v>
       </c>
       <c r="F8" t="n">
-        <v>711918</v>
+        <v>28202</v>
       </c>
       <c r="G8" t="n">
-        <v>209766</v>
+        <v>23276</v>
       </c>
       <c r="H8" t="n">
-        <v>12152</v>
+        <v>742</v>
       </c>
       <c r="I8" t="n">
-        <v>202644</v>
+        <v>182</v>
       </c>
       <c r="J8" t="n">
-        <v>1373</v>
+        <v>182</v>
       </c>
       <c r="K8" t="n">
-        <v>285983</v>
+        <v>3820</v>
       </c>
       <c r="L8" t="n">
-        <v>0.2310029547861961</v>
+        <v>0.3494302767227347</v>
       </c>
       <c r="M8" t="n">
-        <v>0.02363828956904722</v>
+        <v>0.003798155181768855</v>
       </c>
       <c r="N8" t="n">
-        <v>85.90780740919513</v>
+        <v>43.79192546583851</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Republic Airline</t>
+          <t>JetBlue Airways</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>16213</v>
+        <v>212172</v>
       </c>
       <c r="C9" t="n">
-        <v>3224</v>
+        <v>56767</v>
       </c>
       <c r="D9" t="n">
-        <v>567</v>
+        <v>6302</v>
       </c>
       <c r="E9" t="n">
-        <v>25</v>
+        <v>655</v>
       </c>
       <c r="F9" t="n">
-        <v>237421</v>
+        <v>4798379</v>
       </c>
       <c r="G9" t="n">
-        <v>51875</v>
+        <v>1751727</v>
       </c>
       <c r="H9" t="n">
-        <v>14970</v>
+        <v>105335</v>
       </c>
       <c r="I9" t="n">
-        <v>100280</v>
+        <v>894817</v>
       </c>
       <c r="J9" t="n">
-        <v>443</v>
+        <v>8785</v>
       </c>
       <c r="K9" t="n">
-        <v>69853</v>
+        <v>2037715</v>
       </c>
       <c r="L9" t="n">
-        <v>0.1988527724665392</v>
+        <v>0.267551797598175</v>
       </c>
       <c r="M9" t="n">
-        <v>0.03497193610065996</v>
+        <v>0.02970231698810399</v>
       </c>
       <c r="N9" t="n">
-        <v>73.64174937965261</v>
+        <v>84.5276128736766</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SkyWest Airlines</t>
+          <t>Piedmont Airlines</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>575</v>
+        <v>8</v>
       </c>
       <c r="C10" t="n">
-        <v>137</v>
+        <v>1</v>
       </c>
       <c r="D10" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>8466</v>
+        <v>22</v>
       </c>
       <c r="G10" t="n">
-        <v>4732</v>
+        <v>22</v>
       </c>
       <c r="H10" t="n">
-        <v>1243</v>
+        <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>2491</v>
+        <v>0</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -893,13 +893,151 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>0.2382608695652174</v>
+        <v>0.125</v>
       </c>
       <c r="M10" t="n">
-        <v>0.01217391304347826</v>
+        <v>0.375</v>
       </c>
       <c r="N10" t="n">
-        <v>61.7956204379562</v>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Republic Airline</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>82768</v>
+      </c>
+      <c r="C11" t="n">
+        <v>13465</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2585</v>
+      </c>
+      <c r="E11" t="n">
+        <v>132</v>
+      </c>
+      <c r="F11" t="n">
+        <v>911877</v>
+      </c>
+      <c r="G11" t="n">
+        <v>239676</v>
+      </c>
+      <c r="H11" t="n">
+        <v>60116</v>
+      </c>
+      <c r="I11" t="n">
+        <v>355334</v>
+      </c>
+      <c r="J11" t="n">
+        <v>1105</v>
+      </c>
+      <c r="K11" t="n">
+        <v>255646</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.1626836458534699</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0.03123187705393389</v>
+      </c>
+      <c r="N11" t="n">
+        <v>67.72202005198663</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>SkyWest Airlines</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>8109</v>
+      </c>
+      <c r="C12" t="n">
+        <v>1747</v>
+      </c>
+      <c r="D12" t="n">
+        <v>234</v>
+      </c>
+      <c r="E12" t="n">
+        <v>12</v>
+      </c>
+      <c r="F12" t="n">
+        <v>140810</v>
+      </c>
+      <c r="G12" t="n">
+        <v>83508</v>
+      </c>
+      <c r="H12" t="n">
+        <v>31424</v>
+      </c>
+      <c r="I12" t="n">
+        <v>25496</v>
+      </c>
+      <c r="J12" t="n">
+        <v>367</v>
+      </c>
+      <c r="K12" t="n">
+        <v>15</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0.2154396349734863</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0.02885682574916759</v>
+      </c>
+      <c r="N12" t="n">
+        <v>80.60103033772181</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>United Airlines</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>2141</v>
+      </c>
+      <c r="C13" t="n">
+        <v>392</v>
+      </c>
+      <c r="D13" t="n">
+        <v>46</v>
+      </c>
+      <c r="E13" t="n">
+        <v>10</v>
+      </c>
+      <c r="F13" t="n">
+        <v>28561</v>
+      </c>
+      <c r="G13" t="n">
+        <v>12573</v>
+      </c>
+      <c r="H13" t="n">
+        <v>100</v>
+      </c>
+      <c r="I13" t="n">
+        <v>7707</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="n">
+        <v>8181</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0.1830920130780009</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0.02148528724894909</v>
+      </c>
+      <c r="N13" t="n">
+        <v>72.85969387755102</v>
       </c>
     </row>
   </sheetData>

</xml_diff>